<commit_message>
fix: set User Name (email) column to email only in DPL account export
</commit_message>
<xml_diff>
--- a/Daftar_Akun_Login_DPL.xlsx
+++ b/Daftar_Akun_Login_DPL.xlsx
@@ -23,7 +23,7 @@
     <t>Portal Sistem: https://ppl.febuniku.dpdns.org/login | Tahun Akademik 2026/2027</t>
   </si>
   <si>
-    <t>PETUNJUK: Login dapat menggunakan "Username" atau "Email". Password default awal untuk seluruh DPL adalah "FEB_Tangguh".</t>
+    <t>PETUNJUK: DPL dapat login menggunakan "Username" atau "Email". Password default awal untuk seluruh DPL adalah "FEB_Tangguh".</t>
   </si>
   <si>
     <t>No</t>
@@ -50,7 +50,7 @@
     <t>Adi Muhamad Muhsidi, S.SI. M.Kom.</t>
   </si>
   <si>
-    <t>DPL_PPL34 (dpl_ppl34@uniku.ac.id)</t>
+    <t>dpl_ppl34@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL34</t>
@@ -68,7 +68,7 @@
     <t>Amir Hamzah, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL39 (dpl_ppl39@uniku.ac.id)</t>
+    <t>dpl_ppl39@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL39</t>
@@ -80,7 +80,7 @@
     <t>Arief Nurhandika, S.E., M.Ak</t>
   </si>
   <si>
-    <t>DPL_PPL21 (dpl_ppl21@uniku.ac.id)</t>
+    <t>dpl_ppl21@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL21</t>
@@ -92,7 +92,7 @@
     <t>Arief Surya Lesmana, S.Stat., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL26 (dpl_ppl26@uniku.ac.id)</t>
+    <t>dpl_ppl26@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL26</t>
@@ -104,7 +104,7 @@
     <t>Aris Budiman, M.Pd., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL38 (dpl_ppl38@uniku.ac.id)</t>
+    <t>dpl_ppl38@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL38</t>
@@ -116,7 +116,7 @@
     <t>Chintia Fitriani, S.E., M.Ak</t>
   </si>
   <si>
-    <t>DPL_PPL07 (dpl_ppl07@uniku.ac.id)</t>
+    <t>dpl_ppl07@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL07</t>
@@ -128,7 +128,7 @@
     <t>Dadang Suhendar, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL06 (dpl_ppl06@uniku.ac.id)</t>
+    <t>dpl_ppl06@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL06</t>
@@ -140,7 +140,7 @@
     <t>Dendi Purnama, SE., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL41 (dpl_ppl41@uniku.ac.id)</t>
+    <t>dpl_ppl41@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL41</t>
@@ -152,7 +152,7 @@
     <t>Deri Prayudi, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL25 (dpl_ppl25@uniku.ac.id)</t>
+    <t>dpl_ppl25@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL25</t>
@@ -164,7 +164,7 @@
     <t>Dodi, S.Pd., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL23 (dpl_ppl23@uniku.ac.id)</t>
+    <t>dpl_ppl23@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL23</t>
@@ -176,7 +176,7 @@
     <t>Dr. Dadang Suhardi, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL13 (dpl_ppl13@uniku.ac.id)</t>
+    <t>dpl_ppl13@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL13</t>
@@ -188,7 +188,7 @@
     <t>Dr. Dede Djuniardi, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL01 (dpl_ppl01@uniku.ac.id)</t>
+    <t>dpl_ppl01@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL01</t>
@@ -200,7 +200,7 @@
     <t>Dr. Drs. Herma Wiharno, M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL20 (dpl_ppl20@uniku.ac.id)</t>
+    <t>dpl_ppl20@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL20</t>
@@ -212,7 +212,7 @@
     <t>Dr. Ilham Akbar, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL09 (dpl_ppl09@uniku.ac.id)</t>
+    <t>dpl_ppl09@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL09</t>
@@ -224,7 +224,7 @@
     <t>Dr. Iqbal Arraniri, S.E.I., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL10 (dpl_ppl10@uniku.ac.id)</t>
+    <t>dpl_ppl10@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL10</t>
@@ -236,7 +236,7 @@
     <t>Dr. Lili Karmela Fitriani, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL04 (dpl_ppl04@uniku.ac.id)</t>
+    <t>dpl_ppl04@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL04</t>
@@ -248,7 +248,7 @@
     <t>Dr. Munir Nur Komarudin, S.Pd., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL08 (dpl_ppl08@uniku.ac.id)</t>
+    <t>dpl_ppl08@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL08</t>
@@ -260,7 +260,7 @@
     <t>Dr. Neni Nurhayati, S.E., M.Si., Ak., C.A.</t>
   </si>
   <si>
-    <t>DPL_PPL12 (dpl_ppl12@uniku.ac.id)</t>
+    <t>dpl_ppl12@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL12</t>
@@ -272,7 +272,7 @@
     <t>Dr. Rina Masruroh, S.E., ME.Sy</t>
   </si>
   <si>
-    <t>DPL_PPL24 (dpl_ppl24@uniku.ac.id)</t>
+    <t>dpl_ppl24@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL24</t>
@@ -284,7 +284,7 @@
     <t>Dr. Tatang Rois, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL17 (dpl_ppl17@uniku.ac.id)</t>
+    <t>dpl_ppl17@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL17</t>
@@ -296,7 +296,7 @@
     <t>Dr. Yaneri Elfa K. R., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL11 (dpl_ppl11@uniku.ac.id)</t>
+    <t>dpl_ppl11@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL11</t>
@@ -308,7 +308,7 @@
     <t>Dr. Yasir Maulana</t>
   </si>
   <si>
-    <t>DPL_PPL33 (dpl_ppl33@uniku.ac.id)</t>
+    <t>dpl_ppl33@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL33</t>
@@ -320,7 +320,7 @@
     <t>Enung Nurhayati S.E., M.Si., Ak., CA.</t>
   </si>
   <si>
-    <t>DPL_PPL27 (dpl_ppl27@uniku.ac.id)</t>
+    <t>dpl_ppl27@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL27</t>
@@ -332,7 +332,7 @@
     <t>Faishal Rahimi, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL16 (dpl_ppl16@uniku.ac.id)</t>
+    <t>dpl_ppl16@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL16</t>
@@ -344,7 +344,7 @@
     <t>Hadi Satria Ganefi, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL15 (dpl_ppl15@uniku.ac.id)</t>
+    <t>dpl_ppl15@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL15</t>
@@ -356,7 +356,7 @@
     <t>Iman Teguh, S.E., M.Acc</t>
   </si>
   <si>
-    <t>DPL_PPL22 (dpl_ppl22@uniku.ac.id)</t>
+    <t>dpl_ppl22@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL22</t>
@@ -368,7 +368,7 @@
     <t>Januar Habibi Mahsyar, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL35 (dpl_ppl35@uniku.ac.id)</t>
+    <t>dpl_ppl35@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL35</t>
@@ -380,7 +380,7 @@
     <t>Lia Dwi Martika, S.E., M.Si.</t>
   </si>
   <si>
-    <t>DPL_PPL14 (dpl_ppl14@uniku.ac.id)</t>
+    <t>dpl_ppl14@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL14</t>
@@ -392,7 +392,7 @@
     <t>Micki Watulandi, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL19 (dpl_ppl19@uniku.ac.id)</t>
+    <t>dpl_ppl19@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL19</t>
@@ -404,7 +404,7 @@
     <t>Neng Evi kartika, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL32 (dpl_ppl32@uniku.ac.id)</t>
+    <t>dpl_ppl32@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL32</t>
@@ -416,7 +416,7 @@
     <t>Nurul Siti Jahidah, S.P., M.E</t>
   </si>
   <si>
-    <t>DPL_PPL36 (dpl_ppl36@uniku.ac.id)</t>
+    <t>dpl_ppl36@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL36</t>
@@ -428,7 +428,7 @@
     <t>Oktaviani Rita Puspasari, S.E., M.Si, Ak, CA</t>
   </si>
   <si>
-    <t>DPL_PPL29 (dpl_ppl29@uniku.ac.id)</t>
+    <t>dpl_ppl29@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL29</t>
@@ -440,7 +440,7 @@
     <t>Prof. Dr. Dikdik Harjadi, S.E., M.Si</t>
   </si>
   <si>
-    <t>DPL_PPL28 (dpl_ppl28@uniku.ac.id)</t>
+    <t>dpl_ppl28@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL28</t>
@@ -452,7 +452,7 @@
     <t>Qona'ah El Hasan, S.Kom.M.Kom.</t>
   </si>
   <si>
-    <t>DPL_PPL30 (dpl_ppl30@uniku.ac.id)</t>
+    <t>dpl_ppl30@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL30</t>
@@ -464,7 +464,7 @@
     <t>Rizky Indrawan, S.E., M.Ak., Ak., C.A.</t>
   </si>
   <si>
-    <t>DPL_PPL03 (dpl_ppl03@uniku.ac.id)</t>
+    <t>dpl_ppl03@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL03</t>
@@ -476,7 +476,7 @@
     <t>Syahrul Syarifudin, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL31 (dpl_ppl31@uniku.ac.id)</t>
+    <t>dpl_ppl31@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL31</t>
@@ -488,7 +488,7 @@
     <t>Wachjuni, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL05 (dpl_ppl05@uniku.ac.id)</t>
+    <t>dpl_ppl05@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL05</t>
@@ -500,7 +500,7 @@
     <t>Wely Hadi Gunawan, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL18 (dpl_ppl18@uniku.ac.id)</t>
+    <t>dpl_ppl18@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL18</t>
@@ -512,7 +512,7 @@
     <t>Winda Oktaviani, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL40 (dpl_ppl40@uniku.ac.id)</t>
+    <t>dpl_ppl40@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL40</t>
@@ -524,7 +524,7 @@
     <t>Yayan Sopyan, S.Kom., M.Kom</t>
   </si>
   <si>
-    <t>DPL_PPL37 (dpl_ppl37@uniku.ac.id)</t>
+    <t>dpl_ppl37@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL37</t>
@@ -536,7 +536,7 @@
     <t>Yudi Febriansyah, S.E., M.M.</t>
   </si>
   <si>
-    <t>DPL_PPL02 (dpl_ppl02@uniku.ac.id)</t>
+    <t>dpl_ppl02@uniku.ac.id</t>
   </si>
   <si>
     <t>DPL_PPL02</t>
@@ -991,7 +991,7 @@
   <cols>
     <col min="1" max="1" width="5.713" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="52.987" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="25.851" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="16.282" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="90.692" bestFit="true" customWidth="true" style="0"/>

</xml_diff>

<commit_message>
feat: tambah data MBKM (76 mahasiswa, 13 kelompok MBKM, mitra MBKM, dan 2 DPL baru)
</commit_message>
<xml_diff>
--- a/Daftar_Akun_Login_DPL.xlsx
+++ b/Daftar_Akun_Login_DPL.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="184">
   <si>
     <t>DAFTAR AKUN AKSES LOGIN DOSEN PEMBIMBING LAPANGAN (DPL) PPL FEB UNIKU</t>
   </si>
@@ -74,7 +74,7 @@
     <t>DPL_PPL39</t>
   </si>
   <si>
-    <t>KELOMPOK 72</t>
+    <t>KELOMPOK 72, KELOMPOK MBKM - Amir Hamzah</t>
   </si>
   <si>
     <t>Arief Nurhandika, S.E., M.Ak</t>
@@ -146,7 +146,7 @@
     <t>DPL_PPL41</t>
   </si>
   <si>
-    <t>KELOMPOK 78</t>
+    <t>KELOMPOK 78, KELOMPOK MBKM - Dendi Purnama</t>
   </si>
   <si>
     <t>Deri Prayudi, S.E., M.M.</t>
@@ -254,7 +254,7 @@
     <t>DPL_PPL08</t>
   </si>
   <si>
-    <t>KELOMPOK 36, KELOMPOK 53, KELOMPOK 76</t>
+    <t>KELOMPOK 36, KELOMPOK 53, KELOMPOK 76, KELOMPOK MBKM - Dr. Munir Nur Komarudin</t>
   </si>
   <si>
     <t>Dr. Neni Nurhayati, S.E., M.Si., Ak., C.A.</t>
@@ -326,7 +326,7 @@
     <t>DPL_PPL27</t>
   </si>
   <si>
-    <t>KELOMPOK 38, KELOMPOK 62, KELOMPOK 69, KELOMPOK 74</t>
+    <t>KELOMPOK 38, KELOMPOK 62, KELOMPOK 69, KELOMPOK 74, KELOMPOK MBKM - Enung Nurhayati</t>
   </si>
   <si>
     <t>Faishal Rahimi, S.E., M.M.</t>
@@ -422,7 +422,7 @@
     <t>DPL_PPL36</t>
   </si>
   <si>
-    <t>KELOMPOK 63, KELOMPOK 65</t>
+    <t>KELOMPOK 63, KELOMPOK 65, KELOMPOK MBKM - Nurul Siti Jahidah</t>
   </si>
   <si>
     <t>Oktaviani Rita Puspasari, S.E., M.Si, Ak, CA</t>
@@ -434,7 +434,7 @@
     <t>DPL_PPL29</t>
   </si>
   <si>
-    <t>KELOMPOK 41, KELOMPOK 43</t>
+    <t>KELOMPOK 41, KELOMPOK 43, KELOMPOK MBKM - Oktaviani Rita Puspasari</t>
   </si>
   <si>
     <t>Prof. Dr. Dikdik Harjadi, S.E., M.Si</t>
@@ -473,6 +473,18 @@
     <t>KELOMPOK 03, KELOMPOK 14, KELOMPOK 24</t>
   </si>
   <si>
+    <t>Siti Nuke Nurfatimah, M.Sc</t>
+  </si>
+  <si>
+    <t>dpl_ppl42@uniku.ac.id</t>
+  </si>
+  <si>
+    <t>DPL_PPL42</t>
+  </si>
+  <si>
+    <t>KELOMPOK MBKM - Siti Nuke Nurfatimah</t>
+  </si>
+  <si>
     <t>Syahrul Syarifudin, S.E., M.M.</t>
   </si>
   <si>
@@ -482,7 +494,19 @@
     <t>DPL_PPL31</t>
   </si>
   <si>
-    <t>KELOMPOK 45</t>
+    <t>KELOMPOK 45, KELOMPOK MBKM - Syahrul Syarifudin</t>
+  </si>
+  <si>
+    <t>Teti Rahmawati, M.Si., Ak., CA</t>
+  </si>
+  <si>
+    <t>dpl_ppl43@uniku.ac.id</t>
+  </si>
+  <si>
+    <t>DPL_PPL43</t>
+  </si>
+  <si>
+    <t>KELOMPOK MBKM - Teti Rahmawati</t>
   </si>
   <si>
     <t>Wachjuni, S.E., M.M.</t>
@@ -494,7 +518,7 @@
     <t>DPL_PPL05</t>
   </si>
   <si>
-    <t>KELOMPOK 05, KELOMPOK 32, KELOMPOK 61</t>
+    <t>KELOMPOK 05, KELOMPOK 32, KELOMPOK 61, KELOMPOK MBKM - Wachjuni</t>
   </si>
   <si>
     <t>Wely Hadi Gunawan, S.E., M.M.</t>
@@ -506,7 +530,7 @@
     <t>DPL_PPL18</t>
   </si>
   <si>
-    <t>KELOMPOK 22</t>
+    <t>KELOMPOK 22, KELOMPOK MBKM - Wely Hadi Gunawan</t>
   </si>
   <si>
     <t>Winda Oktaviani, S.E., M.M.</t>
@@ -518,7 +542,7 @@
     <t>DPL_PPL40</t>
   </si>
   <si>
-    <t>KELOMPOK 77</t>
+    <t>KELOMPOK 77, KELOMPOK MBKM - Winda Oktaviani</t>
   </si>
   <si>
     <t>Yayan Sopyan, S.Kom., M.Kom</t>
@@ -542,7 +566,7 @@
     <t>DPL_PPL02</t>
   </si>
   <si>
-    <t>KELOMPOK 02</t>
+    <t>KELOMPOK 02, KELOMPOK MBKM - Yudi Febriansyah</t>
   </si>
 </sst>
 </file>
@@ -986,7 +1010,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="5.713" bestFit="true" customWidth="true" style="0"/>
@@ -994,7 +1018,7 @@
     <col min="3" max="3" width="25.851" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="16.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="90.692" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="98.976" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="45.846" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
@@ -1976,6 +2000,52 @@
         <v>175</v>
       </c>
       <c r="G47" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="6">
+        <v>42</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="5">
+        <v>43</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G49" s="5" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>